<commit_message>
DONE:I have completed the data import, cleaning, and preprocessing. FEAT: I created the prediction using Prophet in a modularized way, allowing it to be applied to any result, with configurable risk limits and time horizons.
</commit_message>
<xml_diff>
--- a/source/doc/Dicionario_Dados.xlsx
+++ b/source/doc/Dicionario_Dados.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\Project_Capstone\source\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{745F366F-B11D-4237-B932-4AD831D563EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6E2D46-81BB-4732-AFF2-D2C94DA9A172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{8E3FB131-87B5-4B71-B1AF-28C1D9AD49F1}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="1" xr2:uid="{8E3FB131-87B5-4B71-B1AF-28C1D9AD49F1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Version_Portuguese" sheetId="1" r:id="rId1"/>
+    <sheet name="Version_English" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
   <si>
     <t>Dicionário de Dados</t>
   </si>
@@ -103,6 +104,66 @@
   </si>
   <si>
     <t>Diferença entre receitas e despesas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Name or description of the expense/income.</t>
+  </si>
+  <si>
+    <t>Date or day of the month when the payment is due.</t>
+  </si>
+  <si>
+    <t>Monetary value of the expense or income.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Indicates whether it is an expense or income.</t>
+  </si>
+  <si>
+    <t>Due Date</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Classification of the expense (e.g., Energy, Communication, Taxes).</t>
+  </si>
+  <si>
+    <t>Payment Method</t>
+  </si>
+  <si>
+    <t>Payment method (e.g., PIX, bank slip, automatic debit).</t>
+  </si>
+  <si>
+    <t>Seasonality</t>
+  </si>
+  <si>
+    <t>Estimated value to represent periodic variation (exclusive field for September).</t>
+  </si>
+  <si>
+    <t>Total Income</t>
+  </si>
+  <si>
+    <t>Total amount of money received during the month.</t>
+  </si>
+  <si>
+    <t>Total Expenses</t>
+  </si>
+  <si>
+    <t>Sum of all financial outflows for the month.</t>
+  </si>
+  <si>
+    <t>Balance</t>
+  </si>
+  <si>
+    <t>Difference between income and expenses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dataset Dicionary </t>
   </si>
 </sst>
 </file>
@@ -156,7 +217,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -189,10 +268,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F3245BE-87C5-406D-AA7A-B66DACB4DC89}" name="Tabela1" displayName="Tabela1" ref="A3:B13" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F3245BE-87C5-406D-AA7A-B66DACB4DC89}" name="Tabela1" displayName="Tabela1" ref="A3:B13" totalsRowShown="0" headerRowDxfId="1">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{CDBCFAC4-8A62-4C9C-AFE9-436BD5F0AC38}" name="Variável"/>
     <tableColumn id="2" xr3:uid="{E66AE5BC-B39E-4C3C-A378-AEC618343F29}" name="Descrição"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C63AF176-5370-4B10-8281-FB5BE735F072}" name="Tabela13" displayName="Tabela13" ref="B4:C14" totalsRowShown="0" headerRowDxfId="0">
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{CC542D73-F2E3-4ED1-AA78-57E2DFB77FA9}" name="Variável"/>
+    <tableColumn id="2" xr3:uid="{F74F0EBB-2FF8-4757-827B-B2D25F29EF93}" name="Descrição"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -622,4 +711,115 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF5A689F-58FA-4223-A274-0FB662DBACFE}">
+  <dimension ref="B2:C14"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="66.73046875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
FEAT:FEAT: Importing essential libraries for forecasting with Prophet and data manipulation
</commit_message>
<xml_diff>
--- a/source/doc/Dicionario_Dados.xlsx
+++ b/source/doc/Dicionario_Dados.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\Project_Capstone\source\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6E2D46-81BB-4732-AFF2-D2C94DA9A172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1453120-F27B-4E98-953B-2D6E3AD1E9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" activeTab="1" xr2:uid="{8E3FB131-87B5-4B71-B1AF-28C1D9AD49F1}"/>
+    <workbookView xWindow="-38520" yWindow="7185" windowWidth="38640" windowHeight="21120" xr2:uid="{8E3FB131-87B5-4B71-B1AF-28C1D9AD49F1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Version_Portuguese" sheetId="1" r:id="rId1"/>
-    <sheet name="Version_English" sheetId="2" r:id="rId2"/>
+    <sheet name="Portuguese_Dado_bruto" sheetId="1" r:id="rId1"/>
+    <sheet name="English_ raw_data" sheetId="2" r:id="rId2"/>
+    <sheet name="Portuguese_ Consolidate_data" sheetId="4" r:id="rId3"/>
+    <sheet name="English_ Consolidate_data" sheetId="5" r:id="rId4"/>
+    <sheet name="English_ Prophet Forecast Outp " sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="135">
   <si>
     <t>Dicionário de Dados</t>
   </si>
@@ -164,6 +167,282 @@
   </si>
   <si>
     <t xml:space="preserve">Dataset Dicionary </t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>mes_ano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Mês e ano da referência no formato AAAA-MM.</t>
+  </si>
+  <si>
+    <t>Valor total de receita obtida no mês.</t>
+  </si>
+  <si>
+    <t>receita_do_mes</t>
+  </si>
+  <si>
+    <t>despesa_total</t>
+  </si>
+  <si>
+    <t>Soma total das despesas ocorridas no mês.</t>
+  </si>
+  <si>
+    <t>lucro_bruto</t>
+  </si>
+  <si>
+    <t>Receita do mês menos a despesa total (lucro antes de impostos).</t>
+  </si>
+  <si>
+    <t>ds</t>
+  </si>
+  <si>
+    <t>Data no formato completo YYYY-MM-DD HH:MM:SS, usada para modelos de série temporal (ex: Prophet).</t>
+  </si>
+  <si>
+    <t>ano</t>
+  </si>
+  <si>
+    <t>Ano extraído da data.</t>
+  </si>
+  <si>
+    <t>mês</t>
+  </si>
+  <si>
+    <t>Mês numérico extraído da data.</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>Variável de valor previsto pelo modelo Prophet (valor de referência da previsão).</t>
+  </si>
+  <si>
+    <t>variacao_mensal</t>
+  </si>
+  <si>
+    <t>Variação percentual do lucro previsto em relação ao mês anterior.</t>
+  </si>
+  <si>
+    <t>despesas_acumulada</t>
+  </si>
+  <si>
+    <t>Soma acumulada das despesas ao longo dos meses.</t>
+  </si>
+  <si>
+    <t>lucro_acumulado</t>
+  </si>
+  <si>
+    <t>margem_de_lucro</t>
+  </si>
+  <si>
+    <t>Proporção do lucro em relação à receita (lucro / receita).</t>
+  </si>
+  <si>
+    <t>alerta_risco</t>
+  </si>
+  <si>
+    <t>Indicador de risco baseado em regras definidas para a margem de lucro ou variação — valores como ok ou risco.</t>
+  </si>
+  <si>
+    <t>Month and year in the format YYYY-MM.</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Desciption</t>
+  </si>
+  <si>
+    <t>month_year</t>
+  </si>
+  <si>
+    <t>monthly_revenue</t>
+  </si>
+  <si>
+    <t>Total revenue generated in the given month.</t>
+  </si>
+  <si>
+    <t>total_expense</t>
+  </si>
+  <si>
+    <t>Total amount of expenses incurred during the month.</t>
+  </si>
+  <si>
+    <t>gross_profit</t>
+  </si>
+  <si>
+    <t>Gross profit (monthly revenue minus total expenses).</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>Full date in the format YYYY-MM-DD HH:MM:SS, used for time series models (e.g., Prophet).</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>Year extracted from the date.</t>
+  </si>
+  <si>
+    <t>Predicted value generated by the Prophet model (forecast target).</t>
+  </si>
+  <si>
+    <t>monthly_variation</t>
+  </si>
+  <si>
+    <t>Monthly percentage change in the predicted profit compared to the previous month.</t>
+  </si>
+  <si>
+    <t>cumulative_expense</t>
+  </si>
+  <si>
+    <t>Cumulative sum of expenses over time.</t>
+  </si>
+  <si>
+    <t>cumulative_profit</t>
+  </si>
+  <si>
+    <t>Cumulative sum of monthly gross profits.</t>
+  </si>
+  <si>
+    <t>risk_alert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Risk alert based on defined rules — e.g., low profit margin (ok or risk).</t>
+  </si>
+  <si>
+    <t>profit_margin</t>
+  </si>
+  <si>
+    <t>Profit margin (profit divided by revenue).</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Data Dictionary – Revenue and Forecast Table</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Dicionário de Dados – Tabela de Receita e Predição</t>
+  </si>
+  <si>
+    <t>Desciption2</t>
+  </si>
+  <si>
+    <t>Forecast date.</t>
+  </si>
+  <si>
+    <t>trend</t>
+  </si>
+  <si>
+    <t>Estimated central trend over time.</t>
+  </si>
+  <si>
+    <t>yhat_lower</t>
+  </si>
+  <si>
+    <t>Lower bound of the forecast confidence interval.</t>
+  </si>
+  <si>
+    <t>yhat_upper</t>
+  </si>
+  <si>
+    <t>Upper bound of the forecast confidence interval.</t>
+  </si>
+  <si>
+    <t>trend_lower</t>
+  </si>
+  <si>
+    <t>Lower bound of the estimated trend.</t>
+  </si>
+  <si>
+    <t>trend_upper</t>
+  </si>
+  <si>
+    <t>Upper bound of the estimated trend</t>
+  </si>
+  <si>
+    <t>additive_terms</t>
+  </si>
+  <si>
+    <t>Additive components applied to the forecast (e.g., seasonality, holidays).</t>
+  </si>
+  <si>
+    <t>additive_terms_lower</t>
+  </si>
+  <si>
+    <t>Lower bound of additive terms.</t>
+  </si>
+  <si>
+    <t>Upper bound of additive terms.</t>
+  </si>
+  <si>
+    <t>additive_terms_upper</t>
+  </si>
+  <si>
+    <t>multiplicative_terms</t>
+  </si>
+  <si>
+    <t>Multiplicative components in the forecast (if applicable).</t>
+  </si>
+  <si>
+    <t>multiplicative_terms_upper</t>
+  </si>
+  <si>
+    <t>Upper bound of multiplicative terms.</t>
+  </si>
+  <si>
+    <t>yhat</t>
+  </si>
+  <si>
+    <t>Forecasted value generated by the Prophet model.</t>
+  </si>
+  <si>
+    <t>Risk classification based on business rules (e.g., sharp drop in prediction).</t>
+  </si>
+  <si>
+    <t>Classificação de risco com base em regras de negócio (ex: queda brusca na previsão).</t>
+  </si>
+  <si>
+    <t>Valor previsto pelo modelo Prophet.	Forec</t>
+  </si>
+  <si>
+    <t>Limite superior dos termos multiplicativos.</t>
+  </si>
+  <si>
+    <t>Limite inferior dos termos multiplicativos.</t>
+  </si>
+  <si>
+    <t>Termos multiplicativos aplicados à previsão (caso o modelo os use)</t>
+  </si>
+  <si>
+    <t>Limite superior dos termos aditivos.</t>
+  </si>
+  <si>
+    <t>Limite inferior dos termos aditivos.</t>
+  </si>
+  <si>
+    <t>Termos aditivos aplicados à previsão. (Ex: sazonalidade, feriados)</t>
+  </si>
+  <si>
+    <t>Limite superior da tendência estimada.</t>
+  </si>
+  <si>
+    <t>Limite inferior da tendência estimada.</t>
+  </si>
+  <si>
+    <t>Limite superior do intervalo de confiança da previsão.</t>
+  </si>
+  <si>
+    <t>Limite inferior do intervalo de confiança da previsão.</t>
+  </si>
+  <si>
+    <t>Tendência central estimada ao longo do tempo.</t>
+  </si>
+  <si>
+    <t>Data da previsão.</t>
   </si>
 </sst>
 </file>
@@ -217,7 +496,61 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -268,7 +601,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F3245BE-87C5-406D-AA7A-B66DACB4DC89}" name="Tabela1" displayName="Tabela1" ref="A3:B13" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F3245BE-87C5-406D-AA7A-B66DACB4DC89}" name="Tabela1" displayName="Tabela1" ref="A3:B13" totalsRowShown="0" headerRowDxfId="4">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{CDBCFAC4-8A62-4C9C-AFE9-436BD5F0AC38}" name="Variável"/>
     <tableColumn id="2" xr3:uid="{E66AE5BC-B39E-4C3C-A378-AEC618343F29}" name="Descrição"/>
@@ -278,10 +611,41 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C63AF176-5370-4B10-8281-FB5BE735F072}" name="Tabela13" displayName="Tabela13" ref="B4:C14" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C63AF176-5370-4B10-8281-FB5BE735F072}" name="Tabela13" displayName="Tabela13" ref="B4:C14" totalsRowShown="0" headerRowDxfId="3">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{CC542D73-F2E3-4ED1-AA78-57E2DFB77FA9}" name="Variável"/>
-    <tableColumn id="2" xr3:uid="{F74F0EBB-2FF8-4757-827B-B2D25F29EF93}" name="Descrição"/>
+    <tableColumn id="1" xr3:uid="{CC542D73-F2E3-4ED1-AA78-57E2DFB77FA9}" name="Column"/>
+    <tableColumn id="2" xr3:uid="{F74F0EBB-2FF8-4757-827B-B2D25F29EF93}" name="Description"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6DB57E70-6583-46DA-A9AF-D523F1F7530E}" name="Tabela134" displayName="Tabela134" ref="B4:C22" totalsRowShown="0" headerRowDxfId="2">
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{E325573C-C9E5-4932-A53D-A7310B547FFA}" name="Variável"/>
+    <tableColumn id="2" xr3:uid="{2AD9A425-292B-474C-84A0-36FDC71F369B}" name="Descrição"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{87410F47-2899-4088-83F4-EAE43BDFBB9B}" name="Tabela1345" displayName="Tabela1345" ref="B4:C22" totalsRowShown="0" headerRowDxfId="1">
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{13B31361-A519-4A92-9C3F-2D53F8AF59DE}" name="Column"/>
+    <tableColumn id="2" xr3:uid="{052CB7BD-D916-41E0-A227-59E04E65F6B5}" name="Desciption"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D5116707-A205-4B3F-988C-3A41DAE1F972}" name="Tabela13456" displayName="Tabela13456" ref="B4:D22" totalsRowShown="0" headerRowDxfId="0">
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{B2F39DDB-0D19-4E0C-B849-1E4901E0B735}" name="Column"/>
+    <tableColumn id="3" xr3:uid="{17D8E221-B873-47A4-ADF5-17CF768C225F}" name="Desciption"/>
+    <tableColumn id="2" xr3:uid="{5C97C5F7-48C8-454B-BD4A-E3FA5203D7F4}" name="Desciption2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -730,10 +1094,10 @@
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.45">
@@ -814,6 +1178,466 @@
       </c>
       <c r="C14" t="s">
         <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25AAE01C-F631-4E6B-8106-54EB1CBE7F7D}">
+  <dimension ref="B2:C17"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="20.06640625" customWidth="1"/>
+    <col min="3" max="3" width="94.46484375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC237DD0-351A-4480-94D6-60930F96277B}">
+  <dimension ref="B2:C17"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="20.06640625" customWidth="1"/>
+    <col min="3" max="3" width="94.46484375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B4" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C15" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B16" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B17" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E34124FC-5EED-427D-B9C4-DD74E230729C}">
+  <dimension ref="B2:D18"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="23.1328125" customWidth="1"/>
+    <col min="3" max="3" width="62.06640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="94.46484375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B4" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" t="s">
+        <v>109</v>
+      </c>
+      <c r="D12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B13" t="s">
+        <v>110</v>
+      </c>
+      <c r="C13" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
+        <v>113</v>
+      </c>
+      <c r="C14" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B15" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B16" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" t="s">
+        <v>117</v>
+      </c>
+      <c r="D16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B17" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>